<commit_message>
Feat : Added Empty and incorrect password validation via Excel file
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/testdata.xlsx
+++ b/src/test/resources/testdata/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\testdataexcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A7F7B99-B05D-4C83-BBE4-2E0356923ADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DB55BE8-2589-420E-9783-B6B3BBAFC9A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,6 +17,7 @@
     <sheet name="JoinNowPasswords" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="19">
   <si>
     <t>Email</t>
   </si>
@@ -523,22 +524,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77D7DB55-B4C2-437A-AF8E-921335179FD0}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.5546875" customWidth="1"/>
     <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>13</v>
       </c>
       <c r="B1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -546,7 +551,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -554,7 +559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -562,7 +567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -570,7 +575,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>18</v>
       </c>

</xml_diff>